<commit_message>
Reconcile existing assets and add payment planner and verified assistance routes
</commit_message>
<xml_diff>
--- a/docs/continuity/Civic_Continuum_Startup_Budget_2026-10-18.xlsx
+++ b/docs/continuity/Civic_Continuum_Startup_Budget_2026-10-18.xlsx
@@ -2,8 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="1" r:id="R9bce90eda17740f2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cost register" sheetId="2" r:id="R8b00dbee37814c93"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="1" r:id="R2cb8ae70b2f34eb7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cost register" sheetId="2" r:id="R6af89f882e2248f1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pay today" sheetId="3" r:id="Reae23eeab3d14fd7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Help with costs" sheetId="4" r:id="R7375172ae86646db"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -52,7 +54,7 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="6">
+  <x:fills count="9">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -79,6 +81,21 @@
         <x:fgColor rgb="FFFFF7DC"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF243957"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF7DC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF243957"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="1">
     <x:border>
@@ -92,7 +109,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="24">
+  <x:cellXfs count="37">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -135,6 +152,33 @@
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="5" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="201" fontId="5" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -146,7 +190,7 @@
         <x:color rgb="FFA51C30"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFDE1DE"/>
         </x:patternFill>
       </x:fill>
@@ -375,7 +419,7 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="2" t="str">
-        <x:v>Civic Continuum startup budget</x:v>
+        <x:v>Civic Continuum remaining startup budget</x:v>
       </x:c>
       <x:c r="B2" s="1"/>
       <x:c r="C2" s="1"/>
@@ -468,15 +512,15 @@
     </x:row>
     <x:row r="7" ht="30" customHeight="1">
       <x:c r="A7" s="1" t="str">
-        <x:v>Internal operating allowances — NOT QUOTES</x:v>
+        <x:v>Remaining internal allowances — NOT QUOTES</x:v>
       </x:c>
       <x:c r="B7" s="8" t="n">
         <x:f>'Cost register'!H43</x:f>
-        <x:v>2860</x:v>
+        <x:v>2800</x:v>
       </x:c>
       <x:c r="C7" s="8" t="n">
         <x:f>'Cost register'!I43</x:f>
-        <x:v>9800</x:v>
+        <x:v>9500</x:v>
       </x:c>
       <x:c r="D7" s="1"/>
       <x:c r="E7" s="1"/>
@@ -491,15 +535,15 @@
     </x:row>
     <x:row r="8" ht="30" customHeight="1">
       <x:c r="A8" s="12" t="str">
-        <x:v>Defined budget subtotal</x:v>
+        <x:v>Defined remaining-budget subtotal</x:v>
       </x:c>
       <x:c r="B8" s="13" t="n">
         <x:f>'Cost register'!H44</x:f>
-        <x:v>2951.5</x:v>
+        <x:v>2891.5</x:v>
       </x:c>
       <x:c r="C8" s="13" t="n">
         <x:f>'Cost register'!I44</x:f>
-        <x:v>9928</x:v>
+        <x:v>9628</x:v>
       </x:c>
       <x:c r="D8" s="1"/>
       <x:c r="E8" s="1"/>
@@ -537,15 +581,15 @@
     </x:row>
     <x:row r="10" ht="30" customHeight="1">
       <x:c r="A10" s="1" t="str">
-        <x:v>Defined budget with optional LLC</x:v>
+        <x:v>Remaining budget with optional LLC</x:v>
       </x:c>
       <x:c r="B10" s="8" t="n">
         <x:f>'Cost register'!H45</x:f>
-        <x:v>3151.5</x:v>
+        <x:v>3091.5</x:v>
       </x:c>
       <x:c r="C10" s="8" t="n">
         <x:f>'Cost register'!I45</x:f>
-        <x:v>10128</x:v>
+        <x:v>9828</x:v>
       </x:c>
       <x:c r="D10" s="1"/>
       <x:c r="E10" s="1"/>
@@ -628,7 +672,7 @@
     </x:row>
     <x:row r="15" ht="36" customHeight="1">
       <x:c r="A15" s="3" t="str">
-        <x:v>Excluded: taxes, arrears, payment/postage charges, 2027 city renewal, payroll, patents, trademarks, equipment and buyer-specific audits.</x:v>
+        <x:v>Excluded: existing domain purchase, unpriced hosting/renewals, taxes, arrears, payment charges, payroll, IP filings and buyer audits.</x:v>
       </x:c>
       <x:c r="B15" s="3"/>
       <x:c r="C15" s="3"/>
@@ -801,7 +845,7 @@
     </x:row>
     <x:row r="24" ht="36" customHeight="1">
       <x:c r="A24" s="3" t="str">
-        <x:v>$36.50 city fee requires a genuine July 1-or-later start; otherwise $73. Prior years or penalties may add cost.</x:v>
+        <x:v>Already owned: civiccontinuum.org, paid through September 26, 2027. Do not buy again. Renewal price needs a fresh check.</x:v>
       </x:c>
       <x:c r="B24" s="3"/>
       <x:c r="C24" s="3"/>
@@ -818,7 +862,7 @@
     </x:row>
     <x:row r="25" ht="36" customHeight="1">
       <x:c r="A25" s="3" t="str">
-        <x:v>One $50 opening application and one $5 trade name assumed. Check existing registrations before applying or paying.</x:v>
+        <x:v>Opening fees still conditional: $55 state/name + $36.50 or $73 city. Check actual start date and existing licenses first.</x:v>
       </x:c>
       <x:c r="B25" s="3"/>
       <x:c r="C25" s="3"/>
@@ -869,7 +913,7 @@
     </x:row>
     <x:row r="28" ht="36" customHeight="1">
       <x:c r="A28" s="3" t="str">
-        <x:v>Use the Cost register to replace allowances with quotes, change inclusion flags, and review the source and applicability for each item.</x:v>
+        <x:v>Use Pay today with business-designated funds. All fields start blank or unverified; this template authorizes no spending.</x:v>
       </x:c>
       <x:c r="B28" s="3"/>
       <x:c r="C28" s="3"/>
@@ -899,10 +943,12 @@
       <x:c r="L29" s="1"/>
       <x:c r="M29" s="1"/>
     </x:row>
-    <x:row r="30">
-      <x:c r="A30" s="1"/>
-      <x:c r="B30" s="1"/>
-      <x:c r="C30" s="1"/>
+    <x:row r="30" ht="38" customHeight="1">
+      <x:c r="A30" s="3" t="str">
+        <x:v>See Help with costs: free legal/accounting routes, existing coaches and competitive grants. No pending benefit deducted.</x:v>
+      </x:c>
+      <x:c r="B30" s="3"/>
+      <x:c r="C30" s="3"/>
       <x:c r="D30" s="1"/>
       <x:c r="E30" s="1"/>
       <x:c r="F30" s="1"/>
@@ -1224,6 +1270,7 @@
     <x:mergeCell ref="A26:C26"/>
     <x:mergeCell ref="A27:C27"/>
     <x:mergeCell ref="A28:C28"/>
+    <x:mergeCell ref="A30:C30"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -1249,6 +1296,7 @@
     <x:col min="11" max="11" width="25" hidden="0" customWidth="1"/>
     <x:col min="12" max="12" width="85" hidden="0" customWidth="1"/>
     <x:col min="13" max="13" width="85" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="55" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
@@ -1370,6 +1418,9 @@
       <x:c r="M6" s="6" t="str">
         <x:v>Source / checked 2026-10-18</x:v>
       </x:c>
+      <x:c r="N6" s="34" t="str">
+        <x:v>Help to check before paying</x:v>
+      </x:c>
     </x:row>
     <x:row r="7" ht="100" customHeight="1">
       <x:c r="A7" s="19" t="n">
@@ -1411,6 +1462,9 @@
       <x:c r="M7" s="19" t="str">
         <x:v>https://www.irs.gov/businesses/small-businesses-self-employed/get-an-employer-identification-number</x:v>
       </x:c>
+      <x:c r="N7" s="36" t="str">
+        <x:v>Existing EIN; no paid provider needed.</x:v>
+      </x:c>
     </x:row>
     <x:row r="8" ht="100" customHeight="1">
       <x:c r="A8" s="19" t="n">
@@ -1452,6 +1506,9 @@
       <x:c r="M8" s="19" t="str">
         <x:v>https://dor.wa.gov/open-business/apply-business-license/variable-business-license-processing-fees</x:v>
       </x:c>
+      <x:c r="N8" s="36" t="str">
+        <x:v>Juan/SBDC and Lynette/BINW: confirm sequence and fee-assistance referrals. No fee grant verified.</x:v>
+      </x:c>
     </x:row>
     <x:row r="9" ht="100" customHeight="1">
       <x:c r="A9" s="19" t="n">
@@ -1493,6 +1550,9 @@
       <x:c r="M9" s="19" t="str">
         <x:v>https://dor.wa.gov/open-business/business-licensing-and-renewals-faqs</x:v>
       </x:c>
+      <x:c r="N9" s="36" t="str">
+        <x:v>UBI is part of state process, not a separate paid service.</x:v>
+      </x:c>
     </x:row>
     <x:row r="10" ht="100" customHeight="1">
       <x:c r="A10" s="19" t="n">
@@ -1534,6 +1594,9 @@
       <x:c r="M10" s="19" t="str">
         <x:v>https://dor.wa.gov/manage-business/grow-business/register-trade-names</x:v>
       </x:c>
+      <x:c r="N10" s="36" t="str">
+        <x:v>Juan/SBDC: verify existing trade name before paying again.</x:v>
+      </x:c>
     </x:row>
     <x:row r="11" ht="100" customHeight="1">
       <x:c r="A11" s="19" t="n">
@@ -1575,6 +1638,9 @@
       <x:c r="M11" s="19" t="str">
         <x:v>https://dor.wa.gov/manage-business/grow-business/register-trade-names</x:v>
       </x:c>
+      <x:c r="N11" s="36" t="str">
+        <x:v>Register only real trading names; free adviser can help scope.</x:v>
+      </x:c>
     </x:row>
     <x:row r="12" ht="100" customHeight="1">
       <x:c r="A12" s="19" t="n">
@@ -1616,6 +1682,9 @@
       <x:c r="M12" s="19" t="str">
         <x:v>https://www.seattle.gov/city-finance/business-taxes-and-licenses/business-licenses</x:v>
       </x:c>
+      <x:c r="N12" s="36" t="str">
+        <x:v>City License and Tax Administration / SBDC: verify prior license and true start. No waiver assumed.</x:v>
+      </x:c>
     </x:row>
     <x:row r="13" ht="100" customHeight="1">
       <x:c r="A13" s="19" t="n">
@@ -1653,6 +1722,9 @@
       <x:c r="M13" s="19" t="str">
         <x:v>https://www.seattle.gov/city-finance/business-taxes-and-licenses/business-licenses</x:v>
       </x:c>
+      <x:c r="N13" s="36" t="str">
+        <x:v>Check official payment method charges; no subsidy verified.</x:v>
+      </x:c>
     </x:row>
     <x:row r="14" ht="100" customHeight="1">
       <x:c r="A14" s="19" t="n">
@@ -1694,6 +1766,9 @@
       <x:c r="M14" s="19" t="str">
         <x:v>https://www.sos.wa.gov/corporations-charities/frequently-asked-questions-faqs/fee-schedules-priority-services ; https://app.leg.wa.gov/wac/default.aspx?cite=434-112-075</x:v>
       </x:c>
+      <x:c r="N14" s="36" t="str">
+        <x:v>Communities Rise / City OED legal assistance: entity choice and formation help; state fee not waived automatically.</x:v>
+      </x:c>
     </x:row>
     <x:row r="15" ht="100" customHeight="1">
       <x:c r="A15" s="19" t="n">
@@ -1735,6 +1810,9 @@
       <x:c r="M15" s="19" t="str">
         <x:v>https://www.sos.wa.gov/corporations-charities/frequently-asked-questions-faqs/fee-schedules-priority-services</x:v>
       </x:c>
+      <x:c r="N15" s="36" t="str">
+        <x:v>File with formation to avoid deferred-report fee; free legal route for guidance.</x:v>
+      </x:c>
     </x:row>
     <x:row r="16" ht="100" customHeight="1">
       <x:c r="A16" s="19" t="n">
@@ -1776,6 +1854,9 @@
       <x:c r="M16" s="19" t="str">
         <x:v>https://www.sos.wa.gov/corporations-charities/frequently-asked-questions-faqs/fee-schedules-priority-services</x:v>
       </x:c>
+      <x:c r="N16" s="36" t="str">
+        <x:v>No annual-report fee subsidy verified.</x:v>
+      </x:c>
     </x:row>
     <x:row r="17" ht="100" customHeight="1">
       <x:c r="A17" s="19" t="n">
@@ -1813,6 +1894,9 @@
       <x:c r="M17" s="19" t="str">
         <x:v>https://www.sos.wa.gov/corporations-charities/frequently-asked-questions-faqs/contact-info-requirements-updates</x:v>
       </x:c>
+      <x:c r="N17" s="36" t="str">
+        <x:v>Free entity-choice advice may help; commercial agent service not funded/selected.</x:v>
+      </x:c>
     </x:row>
     <x:row r="18" ht="100" customHeight="1">
       <x:c r="A18" s="19" t="n">
@@ -1854,6 +1938,9 @@
       <x:c r="M18" s="19" t="str">
         <x:v>https://dor.wa.gov/open-business/apply-business-license/variable-business-license-processing-fees</x:v>
       </x:c>
+      <x:c r="N18" s="36" t="str">
+        <x:v>Verify applicable endorsements; no automatic annual UBI fee.</x:v>
+      </x:c>
     </x:row>
     <x:row r="19" ht="100" customHeight="1">
       <x:c r="A19" s="19" t="n">
@@ -1895,6 +1982,9 @@
       <x:c r="M19" s="19" t="str">
         <x:v>https://www.fincen.gov/boi</x:v>
       </x:c>
+      <x:c r="N19" s="36" t="str">
+        <x:v>No domestic BOI service purchase needed under current exemption.</x:v>
+      </x:c>
     </x:row>
     <x:row r="20" ht="100" customHeight="1">
       <x:c r="A20" s="19" t="n">
@@ -1936,6 +2026,9 @@
       <x:c r="M20" s="19" t="str">
         <x:v>https://www.insurance.wa.gov/insurance-resources/business-insurance/learn-how-business-insurance-works</x:v>
       </x:c>
+      <x:c r="N20" s="36" t="str">
+        <x:v>No insurance-premium subsidy verified; compare licensed quotes; grant uses need confirmation.</x:v>
+      </x:c>
     </x:row>
     <x:row r="21" ht="100" customHeight="1">
       <x:c r="A21" s="19" t="n">
@@ -1977,6 +2070,9 @@
       <x:c r="M21" s="19" t="str">
         <x:v>https://www.insurance.wa.gov/insurance-resources/business-insurance/learn-how-business-insurance-works</x:v>
       </x:c>
+      <x:c r="N21" s="36" t="str">
+        <x:v>Compare combined tech E&amp;O/cyber quote; no premium subsidy verified.</x:v>
+      </x:c>
     </x:row>
     <x:row r="22" ht="100" customHeight="1">
       <x:c r="A22" s="19" t="n">
@@ -2018,6 +2114,9 @@
       <x:c r="M22" s="19" t="str">
         <x:v>https://www.insurance.wa.gov/insurance-resources/business-insurance/learn-how-business-insurance-works</x:v>
       </x:c>
+      <x:c r="N22" s="36" t="str">
+        <x:v>Avoid duplicate bundled premium; no subsidy verified.</x:v>
+      </x:c>
     </x:row>
     <x:row r="23" ht="100" customHeight="1">
       <x:c r="A23" s="19" t="n">
@@ -2059,6 +2158,9 @@
       <x:c r="M23" s="19" t="str">
         <x:v>https://communities-rise.org/microenterprise-services/small-business-legal-services/</x:v>
       </x:c>
+      <x:c r="N23" s="36" t="str">
+        <x:v>City OED / Communities Rise free legal help if accepted; SPL questions only, no document review.</x:v>
+      </x:c>
     </x:row>
     <x:row r="24" ht="100" customHeight="1">
       <x:c r="A24" s="19" t="n">
@@ -2100,6 +2202,9 @@
       <x:c r="M24" s="19" t="str">
         <x:v>https://dor.wa.gov/taxes-rates/information-technology-services ; https://www.irs.gov/businesses/small-businesses-self-employed/self-employment-tax-social-security-and-medicare-taxes</x:v>
       </x:c>
+      <x:c r="N24" s="36" t="str">
+        <x:v>Seattle ABC accounting help if approved AFTER active Seattle license. Existing coaches free.</x:v>
+      </x:c>
     </x:row>
     <x:row r="25" ht="100" customHeight="1">
       <x:c r="A25" s="19" t="n">
@@ -2141,6 +2246,9 @@
       <x:c r="M25" s="19" t="str">
         <x:v>Internal planning allowance; define scope with prospective customer.</x:v>
       </x:c>
+      <x:c r="N25" s="36" t="str">
+        <x:v>No free independent security/accessibility assessment secured; define scope before quote.</x:v>
+      </x:c>
     </x:row>
     <x:row r="26" ht="100" customHeight="1">
       <x:c r="A26" s="19" t="n">
@@ -2155,32 +2263,31 @@
       <x:c r="D26" s="19" t="str">
         <x:v>12 months</x:v>
       </x:c>
-      <x:c r="E26" s="20" t="n">
-        <x:v>60</x:v>
-      </x:c>
-      <x:c r="F26" s="20" t="n">
-        <x:v>300</x:v>
-      </x:c>
+      <x:c r="E26" s="20"/>
+      <x:c r="F26" s="20"/>
       <x:c r="G26" s="21" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="H26" s="22" t="n">
         <x:f>IF(G26=0,0,IF(ISNUMBER(E26),E26,"Unpriced"))</x:f>
-        <x:v>60</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="I26" s="22" t="n">
         <x:f>IF(G26=0,0,IF(ISNUMBER(F26),F26,"Unpriced"))</x:f>
-        <x:v>300</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="J26" s="23"/>
       <x:c r="K26" s="19" t="str">
-        <x:v>Incremental allowance</x:v>
+        <x:v>Already established; usage unpriced</x:v>
       </x:c>
       <x:c r="L26" s="19" t="str">
-        <x:v>Internal allowance for ongoing business infrastructure. Existing paid subscriptions and actual bills not reconciled. Do not buy duplicate hosting. AI API usage, personal ChatGPT plan, internet and equipment excluded.</x:v>
+        <x:v>civiccontinuum.org receipt confirms $7.98 paid through 2027-09-26. No replacement domain needed. $11.84 was a historical renewal estimate, not a current invoice. Existing contact forwarding, Sites and Cloudflare free-plan record established; current paid usage/add-ons and future renewal costs still unpriced.</x:v>
       </x:c>
       <x:c r="M26" s="19" t="str">
-        <x:v>Internal planning allowance; existing vendor bills needed.</x:v>
+        <x:v>Existing registrar receipt checked 2026-10-18; private evidence retained. No public order/account details.</x:v>
+      </x:c>
+      <x:c r="N26" s="36" t="str">
+        <x:v>Domain/contact/web infrastructure already exists; do not repurchase.</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="100" customHeight="1">
@@ -2219,6 +2326,9 @@
       <x:c r="M27" s="19" t="str">
         <x:v>No bank selected; obtain fee schedule.</x:v>
       </x:c>
+      <x:c r="N27" s="36" t="str">
+        <x:v>No selected account fee or bank subsidy verified.</x:v>
+      </x:c>
     </x:row>
     <x:row r="28" ht="100" customHeight="1">
       <x:c r="A28" s="19" t="n">
@@ -2260,6 +2370,9 @@
       <x:c r="M28" s="19" t="str">
         <x:v>Internal planning allowance.</x:v>
       </x:c>
+      <x:c r="N28" s="36" t="str">
+        <x:v>Seattle ABC branding/marketing support if eligible; use free digital materials first.</x:v>
+      </x:c>
     </x:row>
     <x:row r="29" ht="100" customHeight="1">
       <x:c r="A29" s="19" t="n">
@@ -2301,6 +2414,9 @@
       <x:c r="M29" s="19" t="str">
         <x:v>https://sam.gov/SAM/?PS=BA</x:v>
       </x:c>
+      <x:c r="N29" s="36" t="str">
+        <x:v>Direct SAM/UEI free.</x:v>
+      </x:c>
     </x:row>
     <x:row r="30" ht="100" customHeight="1">
       <x:c r="A30" s="19" t="n">
@@ -2342,6 +2458,9 @@
       <x:c r="M30" s="19" t="str">
         <x:v>https://des.wa.gov/do-business-state/how-work-state/register-bid-opportunities</x:v>
       </x:c>
+      <x:c r="N30" s="36" t="str">
+        <x:v>Official Census classification tools free.</x:v>
+      </x:c>
     </x:row>
     <x:row r="31" ht="100" customHeight="1">
       <x:c r="A31" s="19" t="n">
@@ -2383,6 +2502,9 @@
       <x:c r="M31" s="19" t="str">
         <x:v>https://des.wa.gov/do-business-state/how-work-state/register-bid-opportunities ; https://careerconnectwa.org/apply-for-funding/</x:v>
       </x:c>
+      <x:c r="N31" s="36" t="str">
+        <x:v>Direct WEBS vendor registration free.</x:v>
+      </x:c>
     </x:row>
     <x:row r="32" ht="100" customHeight="1">
       <x:c r="A32" s="19" t="n">
@@ -2424,6 +2546,9 @@
       <x:c r="M32" s="19" t="str">
         <x:v>https://omwbe.wa.gov/certification/certification-fees</x:v>
       </x:c>
+      <x:c r="N32" s="36" t="str">
+        <x:v>Direct OMWBE certification fees waived; verify eligibility.</x:v>
+      </x:c>
     </x:row>
     <x:row r="33" ht="100" customHeight="1">
       <x:c r="A33" s="19" t="n">
@@ -2465,6 +2590,9 @@
       <x:c r="M33" s="19" t="str">
         <x:v>https://www.sba.gov/certifications/</x:v>
       </x:c>
+      <x:c r="N33" s="36" t="str">
+        <x:v>Direct SBA WOSB/EDWOSB route free; avoid unnecessary paid intermediary.</x:v>
+      </x:c>
     </x:row>
     <x:row r="34" ht="100" customHeight="1">
       <x:c r="A34" s="19" t="n">
@@ -2506,6 +2634,9 @@
       <x:c r="M34" s="19" t="str">
         <x:v>https://wsbdc.org/sbdc-services/ ; https://businessimpactnw.org/grow-your-business/coaching/</x:v>
       </x:c>
+      <x:c r="N34" s="36" t="str">
+        <x:v>Existing free Juan/SBDC and Lynette/BINW relationships.</x:v>
+      </x:c>
     </x:row>
     <x:row r="35" ht="100" customHeight="1">
       <x:c r="A35" s="19" t="n">
@@ -2543,6 +2674,9 @@
       <x:c r="M35" s="19" t="str">
         <x:v>https://www.lni.wa.gov/agency/small-business/common-small-business-questions ; https://esd.wa.gov/employer-requirements/quarterly-reports/how-file-your-quarterly-tax-and-wage-reports</x:v>
       </x:c>
+      <x:c r="N35" s="36" t="str">
+        <x:v>Ask advisers about covered workers; payroll taxes/premiums not waived by mentor program.</x:v>
+      </x:c>
     </x:row>
     <x:row r="36" ht="100" customHeight="1">
       <x:c r="A36" s="19" t="n">
@@ -2580,6 +2714,9 @@
       <x:c r="M36" s="19" t="str">
         <x:v>https://studentprivacy.ed.gov/faq/must-school-have-written-agreement-or-contract-community-based-organization-which-it-non ; https://www.hhs.gov/hipaa/for-professionals/faq/are-we-required-to-certify-our-organizations-compliance-with-the-standards/index.html</x:v>
       </x:c>
+      <x:c r="N36" s="36" t="str">
+        <x:v>Buyer-specific requirements; no blanket certification subsidy verified.</x:v>
+      </x:c>
     </x:row>
     <x:row r="37" ht="100" customHeight="1">
       <x:c r="A37" s="19" t="n">
@@ -2621,6 +2758,9 @@
       <x:c r="M37" s="19" t="str">
         <x:v>https://www.uspto.gov/trademarks/trademark-fee-information</x:v>
       </x:c>
+      <x:c r="N37" s="36" t="str">
+        <x:v>Communities Rise may help with trademark legal work if accepted; USPTO fees separate.</x:v>
+      </x:c>
     </x:row>
     <x:row r="38" ht="100" customHeight="1">
       <x:c r="A38" s="19" t="n">
@@ -2662,6 +2802,9 @@
       <x:c r="M38" s="19" t="str">
         <x:v>https://www.uspto.gov/learning-and-resources/fees-and-payment/uspto-fee-schedule</x:v>
       </x:c>
+      <x:c r="N38" s="36" t="str">
+        <x:v>Existing TILE intake acknowledged; attorney services free IF matched, filing fees remain inventor expense.</x:v>
+      </x:c>
     </x:row>
     <x:row r="39" ht="100" customHeight="1">
       <x:c r="A39" s="19" t="n">
@@ -2698,6 +2841,9 @@
       </x:c>
       <x:c r="M39" s="19" t="str">
         <x:v>https://dor.wa.gov/taxes-rates/information-technology-services ; https://seattle.gov/city-finance/business-taxes-and-licenses/business-taxes ; https://www.irs.gov/businesses/small-businesses-self-employed/self-employment-tax-social-security-and-medicare-taxes</x:v>
+      </x:c>
+      <x:c r="N39" s="36" t="str">
+        <x:v>Seattle ABC may help tax/accounting if eligible; tax liabilities not erased by coaching.</x:v>
       </x:c>
     </x:row>
     <x:row r="40">
@@ -2765,11 +2911,11 @@
       <x:c r="G43" s="10"/>
       <x:c r="H43" s="11" t="n">
         <x:f>IF(COUNTIFS($C$7:$C$39,"Reserve",H7:H39,"Unpriced")&gt;0,"Unpriced",SUMIFS(H7:H39,$C$7:$C$39,"Reserve"))</x:f>
-        <x:v>2860</x:v>
+        <x:v>2800</x:v>
       </x:c>
       <x:c r="I43" s="11" t="n">
         <x:f>IF(COUNTIFS($C$7:$C$39,"Reserve",I7:I39,"Unpriced")&gt;0,"Unpriced",SUMIFS(I7:I39,$C$7:$C$39,"Reserve"))</x:f>
-        <x:v>9800</x:v>
+        <x:v>9500</x:v>
       </x:c>
       <x:c r="J43" s="1"/>
       <x:c r="K43" s="1"/>
@@ -2788,11 +2934,11 @@
       <x:c r="G44" s="10"/>
       <x:c r="H44" s="11" t="n">
         <x:f>IF(COUNTIFS(H7:H39,"Unpriced")&gt;0,"Unpriced",SUM(H7:H39))</x:f>
-        <x:v>2951.5</x:v>
+        <x:v>2891.5</x:v>
       </x:c>
       <x:c r="I44" s="11" t="n">
         <x:f>IF(COUNTIFS(I7:I39,"Unpriced")&gt;0,"Unpriced",SUM(I7:I39))</x:f>
-        <x:v>9928</x:v>
+        <x:v>9628</x:v>
       </x:c>
       <x:c r="J44" s="1"/>
       <x:c r="K44" s="1"/>
@@ -2811,11 +2957,11 @@
       <x:c r="G45" s="10"/>
       <x:c r="H45" s="11" t="n">
         <x:f>IF(ISNUMBER(H44),H44+E14,"Unpriced")</x:f>
-        <x:v>3151.5</x:v>
+        <x:v>3091.5</x:v>
       </x:c>
       <x:c r="I45" s="11" t="n">
         <x:f>IF(ISNUMBER(I44),I44+F14,"Unpriced")</x:f>
-        <x:v>10128</x:v>
+        <x:v>9828</x:v>
       </x:c>
       <x:c r="J45" s="1"/>
       <x:c r="K45" s="1"/>
@@ -2915,4 +3061,780 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetPr>
+    <x:tabColor rgb="FF243957"/>
+  </x:sheetPr>
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="40" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="25" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="18" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="18" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="18" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="43" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="1"/>
+      <x:c r="B1" s="1"/>
+      <x:c r="C1" s="1"/>
+      <x:c r="D1" s="1"/>
+      <x:c r="E1" s="1"/>
+      <x:c r="F1" s="1"/>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="2" t="str">
+        <x:v>What can we fund today?</x:v>
+      </x:c>
+      <x:c r="B2" s="1"/>
+      <x:c r="C2" s="1"/>
+      <x:c r="D2" s="1"/>
+      <x:c r="E2" s="1"/>
+      <x:c r="F2" s="1"/>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="1"/>
+      <x:c r="B3" s="1"/>
+      <x:c r="C3" s="1"/>
+      <x:c r="D3" s="1"/>
+      <x:c r="E3" s="1"/>
+      <x:c r="F3" s="1"/>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="1" t="str">
+        <x:v>Business-designated money available</x:v>
+      </x:c>
+      <x:c r="B4" s="30"/>
+      <x:c r="C4" s="1"/>
+      <x:c r="D4" s="1"/>
+      <x:c r="E4" s="1"/>
+      <x:c r="F4" s="1"/>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="1" t="str">
+        <x:v>Amount to keep back</x:v>
+      </x:c>
+      <x:c r="B5" s="30" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C5" s="1"/>
+      <x:c r="D5" s="1"/>
+      <x:c r="E5" s="1"/>
+      <x:c r="F5" s="1"/>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="1" t="str">
+        <x:v>Usable business money</x:v>
+      </x:c>
+      <x:c r="B6" s="8" t="str">
+        <x:f>IF(ISNUMBER(B4),MAX(0,B4-B5),"Enter available amount")</x:f>
+        <x:v>Enter available amount</x:v>
+      </x:c>
+      <x:c r="C6" s="1"/>
+      <x:c r="D6" s="1"/>
+      <x:c r="E6" s="1"/>
+      <x:c r="F6" s="1"/>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="1" t="str">
+        <x:v>Remaining after priority reserves</x:v>
+      </x:c>
+      <x:c r="B7" s="8" t="str">
+        <x:f>IF(ISNUMBER(B6),B6-SUM(D12:D13),"Enter available amount")</x:f>
+        <x:v>Enter available amount</x:v>
+      </x:c>
+      <x:c r="C7" s="1"/>
+      <x:c r="D7" s="1"/>
+      <x:c r="E7" s="1"/>
+      <x:c r="F7" s="1"/>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="1"/>
+      <x:c r="B8" s="1"/>
+      <x:c r="C8" s="1"/>
+      <x:c r="D8" s="1"/>
+      <x:c r="E8" s="1"/>
+      <x:c r="F8" s="1"/>
+    </x:row>
+    <x:row r="9" ht="38" customHeight="1">
+      <x:c r="A9" s="3" t="str">
+        <x:v>Exclude household essentials, sales tax held, refundable customer funds and restricted funds from the amount entered.</x:v>
+      </x:c>
+      <x:c r="B9" s="3"/>
+      <x:c r="C9" s="3"/>
+      <x:c r="D9" s="3"/>
+      <x:c r="E9" s="3"/>
+      <x:c r="F9" s="3"/>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="1"/>
+      <x:c r="B10" s="1"/>
+      <x:c r="C10" s="1"/>
+      <x:c r="D10" s="1"/>
+      <x:c r="E10" s="1"/>
+      <x:c r="F10" s="1"/>
+    </x:row>
+    <x:row r="11" ht="50" customHeight="1">
+      <x:c r="A11" s="25" t="str">
+        <x:v>Priority item</x:v>
+      </x:c>
+      <x:c r="B11" s="25" t="str">
+        <x:v>Fee to reserve</x:v>
+      </x:c>
+      <x:c r="C11" s="25" t="str">
+        <x:v>Records verified 1/0</x:v>
+      </x:c>
+      <x:c r="D11" s="25" t="str">
+        <x:v>Reserved today</x:v>
+      </x:c>
+      <x:c r="E11" s="25" t="str">
+        <x:v>Still needed</x:v>
+      </x:c>
+      <x:c r="F11" s="25" t="str">
+        <x:v>Next action</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="50" customHeight="1">
+      <x:c r="A12" s="3" t="str">
+        <x:v>WA opening + one trade name</x:v>
+      </x:c>
+      <x:c r="B12" s="31" t="n">
+        <x:v>55</x:v>
+      </x:c>
+      <x:c r="C12" s="29" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D12" s="9" t="str">
+        <x:f>IF(ISNUMBER($B$6),MIN($B$6,B12),"Enter amount")</x:f>
+        <x:v>Enter amount</x:v>
+      </x:c>
+      <x:c r="E12" s="9" t="str">
+        <x:f>IF(ISNUMBER(D12),B12-D12,"Enter amount")</x:f>
+        <x:v>Enter amount</x:v>
+      </x:c>
+      <x:c r="F12" s="3" t="str">
+        <x:f>IF(ISNUMBER(D12),IF(E12&gt;0,"Save toward this fee",IF(C12=1,"Review final fee and payment approval","Reserve only; verify existing records")),"Enter business budget first")</x:f>
+        <x:v>Enter business budget first</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="50" customHeight="1">
+      <x:c r="A13" s="3" t="str">
+        <x:v>Seattle first year, conservative</x:v>
+      </x:c>
+      <x:c r="B13" s="31" t="n">
+        <x:v>73</x:v>
+      </x:c>
+      <x:c r="C13" s="29" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D13" s="9" t="str">
+        <x:f>IF(ISNUMBER($B$6),MIN(MAX(0,$B$6-B12),B13),"Enter amount")</x:f>
+        <x:v>Enter amount</x:v>
+      </x:c>
+      <x:c r="E13" s="9" t="str">
+        <x:f>IF(ISNUMBER(D13),B13-D13,"Enter amount")</x:f>
+        <x:v>Enter amount</x:v>
+      </x:c>
+      <x:c r="F13" s="3" t="str">
+        <x:f>IF(ISNUMBER(D13),IF(E13&gt;0,"Save toward this fee",IF(C13=1,"Review final fee and payment approval","Reserve only; verify existing records")),"Enter business budget first")</x:f>
+        <x:v>Enter business budget first</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="1"/>
+      <x:c r="B14" s="1"/>
+      <x:c r="C14" s="1"/>
+      <x:c r="D14" s="1"/>
+      <x:c r="E14" s="1"/>
+      <x:c r="F14" s="1"/>
+    </x:row>
+    <x:row r="15" ht="40" customHeight="1">
+      <x:c r="A15" s="3" t="str">
+        <x:v>This allocates a reserve, not a payment. Government records, actual start date and final transaction charges remain prerequisites.</x:v>
+      </x:c>
+      <x:c r="B15" s="3"/>
+      <x:c r="C15" s="3"/>
+      <x:c r="D15" s="3"/>
+      <x:c r="E15" s="3"/>
+      <x:c r="F15" s="3"/>
+    </x:row>
+    <x:row r="16" ht="40" customHeight="1">
+      <x:c r="A16" s="3" t="str">
+        <x:v>The $55 state/name amount is one combined application, not two separate payments. Reduce city fee only after half-rate eligibility is verified.</x:v>
+      </x:c>
+      <x:c r="B16" s="3"/>
+      <x:c r="C16" s="3"/>
+      <x:c r="D16" s="3"/>
+      <x:c r="E16" s="3"/>
+      <x:c r="F16" s="3"/>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="1"/>
+      <x:c r="B17" s="1"/>
+      <x:c r="C17" s="1"/>
+      <x:c r="D17" s="1"/>
+      <x:c r="E17" s="1"/>
+      <x:c r="F17" s="1"/>
+    </x:row>
+    <x:row r="18" ht="52" customHeight="1">
+      <x:c r="A18" s="25" t="str">
+        <x:v>Do not repurchase</x:v>
+      </x:c>
+      <x:c r="B18" s="25" t="str">
+        <x:v>Evidence</x:v>
+      </x:c>
+      <x:c r="C18" s="25" t="str">
+        <x:v>Money needed now</x:v>
+      </x:c>
+      <x:c r="D18" s="1"/>
+      <x:c r="E18" s="1"/>
+      <x:c r="F18" s="1"/>
+    </x:row>
+    <x:row r="19" ht="52" customHeight="1">
+      <x:c r="A19" s="3" t="str">
+        <x:v>civiccontinuum.org</x:v>
+      </x:c>
+      <x:c r="B19" s="3" t="str">
+        <x:v>Receipt: paid through 2027-09-26</x:v>
+      </x:c>
+      <x:c r="C19" s="3" t="str">
+        <x:v>No duplicate purchase</x:v>
+      </x:c>
+      <x:c r="D19" s="1"/>
+      <x:c r="E19" s="1"/>
+      <x:c r="F19" s="1"/>
+    </x:row>
+    <x:row r="20" ht="52" customHeight="1">
+      <x:c r="A20" s="3" t="str">
+        <x:v>EIN</x:v>
+      </x:c>
+      <x:c r="B20" s="3" t="str">
+        <x:v>Existing assignment documented</x:v>
+      </x:c>
+      <x:c r="C20" s="3" t="str">
+        <x:v>No duplicate application</x:v>
+      </x:c>
+      <x:c r="D20" s="1"/>
+      <x:c r="E20" s="1"/>
+      <x:c r="F20" s="1"/>
+    </x:row>
+    <x:row r="21" ht="52" customHeight="1">
+      <x:c r="A21" s="3" t="str">
+        <x:v>Contact email and websites</x:v>
+      </x:c>
+      <x:c r="B21" s="3" t="str">
+        <x:v>Existing infrastructure</x:v>
+      </x:c>
+      <x:c r="C21" s="3" t="str">
+        <x:v>No duplicate purchase</x:v>
+      </x:c>
+      <x:c r="D21" s="1"/>
+      <x:c r="E21" s="1"/>
+      <x:c r="F21" s="1"/>
+    </x:row>
+    <x:row r="22" ht="52" customHeight="1">
+      <x:c r="A22" s="3" t="str">
+        <x:v>Insurance and legal review</x:v>
+      </x:c>
+      <x:c r="B22" s="3" t="str">
+        <x:v>No policy / quote verified</x:v>
+      </x:c>
+      <x:c r="C22" s="3" t="str">
+        <x:v>Get scoped quote or free help</x:v>
+      </x:c>
+      <x:c r="D22" s="1"/>
+      <x:c r="E22" s="1"/>
+      <x:c r="F22" s="1"/>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" s="1"/>
+      <x:c r="B23" s="1"/>
+      <x:c r="C23" s="1"/>
+      <x:c r="D23" s="1"/>
+      <x:c r="E23" s="1"/>
+      <x:c r="F23" s="1"/>
+    </x:row>
+    <x:row r="24" ht="40" customHeight="1">
+      <x:c r="A24" s="3" t="str">
+        <x:v>Optional LLC $200 is not automatically allocated. Review structure, agent consent and annual $70 report before choosing it.</x:v>
+      </x:c>
+      <x:c r="B24" s="3"/>
+      <x:c r="C24" s="3"/>
+      <x:c r="D24" s="3"/>
+      <x:c r="E24" s="3"/>
+      <x:c r="F24" s="3"/>
+    </x:row>
+    <x:row r="25" ht="40" customHeight="1">
+      <x:c r="A25" s="3" t="str">
+        <x:v>Before using new money: read the private Money Available Playbook, refresh fees, subtract receipts already paid, and ask only for missing facts.</x:v>
+      </x:c>
+      <x:c r="B25" s="3"/>
+      <x:c r="C25" s="3"/>
+      <x:c r="D25" s="3"/>
+      <x:c r="E25" s="3"/>
+      <x:c r="F25" s="3"/>
+    </x:row>
+    <x:row r="26" ht="40" customHeight="1">
+      <x:c r="A26" s="3" t="str">
+        <x:v>This public template contains no cash balance. Never publish a populated copy, financial account details or private payment receipts.</x:v>
+      </x:c>
+      <x:c r="B26" s="3"/>
+      <x:c r="C26" s="3"/>
+      <x:c r="D26" s="3"/>
+      <x:c r="E26" s="3"/>
+      <x:c r="F26" s="3"/>
+    </x:row>
+    <x:row r="27">
+      <x:c r="A27" s="1"/>
+      <x:c r="B27" s="1"/>
+      <x:c r="C27" s="1"/>
+      <x:c r="D27" s="1"/>
+      <x:c r="E27" s="1"/>
+      <x:c r="F27" s="1"/>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" s="1"/>
+      <x:c r="B28" s="1"/>
+      <x:c r="C28" s="1"/>
+      <x:c r="D28" s="1"/>
+      <x:c r="E28" s="1"/>
+      <x:c r="F28" s="1"/>
+    </x:row>
+    <x:row r="29">
+      <x:c r="A29" s="1"/>
+      <x:c r="B29" s="1"/>
+      <x:c r="C29" s="1"/>
+      <x:c r="D29" s="1"/>
+      <x:c r="E29" s="1"/>
+      <x:c r="F29" s="1"/>
+    </x:row>
+    <x:row r="30">
+      <x:c r="A30" s="1"/>
+      <x:c r="B30" s="1"/>
+      <x:c r="C30" s="1"/>
+      <x:c r="D30" s="1"/>
+      <x:c r="E30" s="1"/>
+      <x:c r="F30" s="1"/>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A9:F9"/>
+    <x:mergeCell ref="A15:F15"/>
+    <x:mergeCell ref="A16:F16"/>
+    <x:mergeCell ref="A24:F24"/>
+    <x:mergeCell ref="A25:F25"/>
+    <x:mergeCell ref="A26:F26"/>
+  </x:mergeCells>
+  <x:dataValidations count="1">
+    <x:dataValidation type="list" sqref="C12:C13">
+      <x:formula1>"0,1"</x:formula1>
+    </x:dataValidation>
+  </x:dataValidations>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetPr>
+    <x:tabColor rgb="FF243957"/>
+  </x:sheetPr>
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="31" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="28" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="28" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="30" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="46" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="46" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="46" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="70" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="1"/>
+      <x:c r="B1" s="1"/>
+      <x:c r="C1" s="1"/>
+      <x:c r="D1" s="1"/>
+      <x:c r="E1" s="1"/>
+      <x:c r="F1" s="1"/>
+      <x:c r="G1" s="1"/>
+      <x:c r="H1" s="1"/>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="2" t="str">
+        <x:v>Programs that may reduce our costs</x:v>
+      </x:c>
+      <x:c r="B2" s="1"/>
+      <x:c r="C2" s="1"/>
+      <x:c r="D2" s="1"/>
+      <x:c r="E2" s="1"/>
+      <x:c r="F2" s="1"/>
+      <x:c r="G2" s="1"/>
+      <x:c r="H2" s="1"/>
+    </x:row>
+    <x:row r="3" ht="32" customHeight="1">
+      <x:c r="A3" s="3" t="str">
+        <x:v>Checked October 18, 2026. Free services and competitive grants are separate. Nothing pending is deducted from the budget.</x:v>
+      </x:c>
+      <x:c r="B3" s="3"/>
+      <x:c r="C3" s="3"/>
+      <x:c r="D3" s="3"/>
+      <x:c r="E3" s="3"/>
+      <x:c r="F3" s="3"/>
+      <x:c r="G3" s="3"/>
+      <x:c r="H3" s="3"/>
+    </x:row>
+    <x:row r="4" ht="32" customHeight="1">
+      <x:c r="A4" s="3" t="str">
+        <x:v>No general license-fee waiver or insurance-premium subsidy verified. No award, enrollment, loan or matching commitment created.</x:v>
+      </x:c>
+      <x:c r="B4" s="3"/>
+      <x:c r="C4" s="3"/>
+      <x:c r="D4" s="3"/>
+      <x:c r="E4" s="3"/>
+      <x:c r="F4" s="3"/>
+      <x:c r="G4" s="3"/>
+      <x:c r="H4" s="3"/>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="1"/>
+      <x:c r="B5" s="1"/>
+      <x:c r="C5" s="1"/>
+      <x:c r="D5" s="1"/>
+      <x:c r="E5" s="1"/>
+      <x:c r="F5" s="1"/>
+      <x:c r="G5" s="1"/>
+      <x:c r="H5" s="1"/>
+    </x:row>
+    <x:row r="6" ht="42" customHeight="1">
+      <x:c r="A6" s="34" t="str">
+        <x:v>Program</x:v>
+      </x:c>
+      <x:c r="B6" s="34" t="str">
+        <x:v>Cost it may help</x:v>
+      </x:c>
+      <x:c r="C6" s="34" t="str">
+        <x:v>Type</x:v>
+      </x:c>
+      <x:c r="D6" s="34" t="str">
+        <x:v>Value / limit</x:v>
+      </x:c>
+      <x:c r="E6" s="34" t="str">
+        <x:v>Eligibility / prerequisite</x:v>
+      </x:c>
+      <x:c r="F6" s="34" t="str">
+        <x:v>Our status</x:v>
+      </x:c>
+      <x:c r="G6" s="34" t="str">
+        <x:v>Next action / restriction</x:v>
+      </x:c>
+      <x:c r="H6" s="34" t="str">
+        <x:v>Official source</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="120" customHeight="1">
+      <x:c r="A7" s="3" t="str">
+        <x:v>Seattle OED legal assistance</x:v>
+      </x:c>
+      <x:c r="B7" s="3" t="str">
+        <x:v>Legal / formation / IP guidance</x:v>
+      </x:c>
+      <x:c r="C7" s="3" t="str">
+        <x:v>Free in-kind service</x:v>
+      </x:c>
+      <x:c r="D7" s="3" t="str">
+        <x:v>Scope approved by provider</x:v>
+      </x:c>
+      <x:c r="E7" s="3" t="str">
+        <x:v>Seattle-based business; capacity and scope approval</x:v>
+      </x:c>
+      <x:c r="F7" s="3" t="str">
+        <x:v>Not enrolled in this task</x:v>
+      </x:c>
+      <x:c r="G7" s="3" t="str">
+        <x:v>Use City intake/referral; distinguish advice from document review</x:v>
+      </x:c>
+      <x:c r="H7" s="3" t="str">
+        <x:v>https://seattle.gov/economic-development/grow-a-business/consulting-services/legal-assistance</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="120" customHeight="1">
+      <x:c r="A8" s="3" t="str">
+        <x:v>Communities Rise direct services</x:v>
+      </x:c>
+      <x:c r="B8" s="3" t="str">
+        <x:v>Contracts, formation, licenses, privacy</x:v>
+      </x:c>
+      <x:c r="C8" s="3" t="str">
+        <x:v>Free if eligible</x:v>
+      </x:c>
+      <x:c r="D8" s="3" t="str">
+        <x:v>Accepted engagement scope</x:v>
+      </x:c>
+      <x:c r="E8" s="3" t="str">
+        <x:v>WA registration, financial eligibility and capacity need confirmation</x:v>
+      </x:c>
+      <x:c r="F8" s="3" t="str">
+        <x:v>Lynette referral requested; not accepted</x:v>
+      </x:c>
+      <x:c r="G8" s="3" t="str">
+        <x:v>Confirm intake and substantive document-review scope; patents excluded</x:v>
+      </x:c>
+      <x:c r="H8" s="3" t="str">
+        <x:v>https://communities-rise.org/microenterprise-services/small-business-legal-services/</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="120" customHeight="1">
+      <x:c r="A9" s="3" t="str">
+        <x:v>Seattle ABC consulting</x:v>
+      </x:c>
+      <x:c r="B9" s="3" t="str">
+        <x:v>Accounting, operations, financial plan, branding</x:v>
+      </x:c>
+      <x:c r="C9" s="3" t="str">
+        <x:v>Free in-kind service</x:v>
+      </x:c>
+      <x:c r="D9" s="3" t="str">
+        <x:v>Up to 10 hours/category; up to 40 total</x:v>
+      </x:c>
+      <x:c r="E9" s="3" t="str">
+        <x:v>Active Seattle license; Seattle location, &lt;=2 locations, &lt;=50 staff, revenue under $5m</x:v>
+      </x:c>
+      <x:c r="F9" s="3" t="str">
+        <x:v>City-license prerequisite unverified</x:v>
+      </x:c>
+      <x:c r="G9" s="3" t="str">
+        <x:v>Apply after license proof; no cash or license-fee reimbursement promised</x:v>
+      </x:c>
+      <x:c r="H9" s="3" t="str">
+        <x:v>https://www.seattle.gov/economic-development/grow-a-business/consulting-services/accounting-and-business-consulting-program</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="120" customHeight="1">
+      <x:c r="A10" s="3" t="str">
+        <x:v>SPL legal / Library to Business</x:v>
+      </x:c>
+      <x:c r="B10" s="3" t="str">
+        <x:v>Legal questions and market research</x:v>
+      </x:c>
+      <x:c r="C10" s="3" t="str">
+        <x:v>Free consultation</x:v>
+      </x:c>
+      <x:c r="D10" s="3" t="str">
+        <x:v>Appointment scope only</x:v>
+      </x:c>
+      <x:c r="E10" s="3" t="str">
+        <x:v>Appointment availability; legal consult does not review documents</x:v>
+      </x:c>
+      <x:c r="F10" s="3" t="str">
+        <x:v>Available route; not booked</x:v>
+      </x:c>
+      <x:c r="G10" s="3" t="str">
+        <x:v>Use for initial questions/research; not substitute for contract redline</x:v>
+      </x:c>
+      <x:c r="H10" s="3" t="str">
+        <x:v>https://www.spl.org/programs-and-services/business-and-nonprofit/make-a-business-appointment/business-appointment-legal-consults</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="120" customHeight="1">
+      <x:c r="A11" s="3" t="str">
+        <x:v>WA TILE Patent Pro Bono</x:v>
+      </x:c>
+      <x:c r="B11" s="3" t="str">
+        <x:v>Patent attorney work</x:v>
+      </x:c>
+      <x:c r="C11" s="3" t="str">
+        <x:v>Free legal service if matched</x:v>
+      </x:c>
+      <x:c r="D11" s="3" t="str">
+        <x:v>Attorney services only</x:v>
+      </x:c>
+      <x:c r="E11" s="3" t="str">
+        <x:v>WA residence, household/asset rules, training, actual invention; matching not guaranteed</x:v>
+      </x:c>
+      <x:c r="F11" s="3" t="str">
+        <x:v>Existing application acknowledged; no attorney match established</x:v>
+      </x:c>
+      <x:c r="G11" s="3" t="str">
+        <x:v>Follow existing intake; inventor still pays USPTO and other out-of-pocket costs</x:v>
+      </x:c>
+      <x:c r="H11" s="3" t="str">
+        <x:v>https://law.seattleu.edu/academics/degree-programs/jd/curriculum/tile/wa-tile-patent-pro-bono-hub/</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="120" customHeight="1">
+      <x:c r="A12" s="3" t="str">
+        <x:v>Verizon Digital Ready / LISC</x:v>
+      </x:c>
+      <x:c r="B12" s="3" t="str">
+        <x:v>Potential business funding</x:v>
+      </x:c>
+      <x:c r="C12" s="3" t="str">
+        <x:v>Competitive cash grant</x:v>
+      </x:c>
+      <x:c r="D12" s="3" t="str">
+        <x:v>$10,000 if awarded</x:v>
+      </x:c>
+      <x:c r="E12" s="3" t="str">
+        <x:v>Two eligible 2026 courses/events by Dec 7; for-profit eligibility; finalist verification</x:v>
+      </x:c>
+      <x:c r="F12" s="3" t="str">
+        <x:v>Candidate only; no application or award verified</x:v>
+      </x:c>
+      <x:c r="G12" s="3" t="str">
+        <x:v>Check existing enrollment/application and data requirements before applying; eligible uses need confirmation</x:v>
+      </x:c>
+      <x:c r="H12" s="3" t="str">
+        <x:v>https://digitalready.verizonwireless.com/funding/details</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="120" customHeight="1">
+      <x:c r="A13" s="3" t="str">
+        <x:v>Awesome Foundation Seattle</x:v>
+      </x:c>
+      <x:c r="B13" s="3" t="str">
+        <x:v>Specific local community-benefit project</x:v>
+      </x:c>
+      <x:c r="C13" s="3" t="str">
+        <x:v>Competitive project grant</x:v>
+      </x:c>
+      <x:c r="D13" s="3" t="str">
+        <x:v>Typically $1,000</x:v>
+      </x:c>
+      <x:c r="E13" s="3" t="str">
+        <x:v>Chapter selects projects; local impact and permitted use need fit</x:v>
+      </x:c>
+      <x:c r="F13" s="3" t="str">
+        <x:v>Candidate only; no award verified</x:v>
+      </x:c>
+      <x:c r="G13" s="3" t="str">
+        <x:v>Propose concrete public-benefit project; don't assume general overhead funded</x:v>
+      </x:c>
+      <x:c r="H13" s="3" t="str">
+        <x:v>https://www.awesomefoundation.org/chapters/seattle</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="120" customHeight="1">
+      <x:c r="A14" s="3" t="str">
+        <x:v>Juan / Washington SBDC</x:v>
+      </x:c>
+      <x:c r="B14" s="3" t="str">
+        <x:v>Licensing sequence and business planning</x:v>
+      </x:c>
+      <x:c r="C14" s="3" t="str">
+        <x:v>Existing no-cost adviser</x:v>
+      </x:c>
+      <x:c r="D14" s="3" t="str">
+        <x:v>Advising, not cash award</x:v>
+      </x:c>
+      <x:c r="E14" s="3" t="str">
+        <x:v>Current client relationship</x:v>
+      </x:c>
+      <x:c r="F14" s="3" t="str">
+        <x:v>Existing relationship</x:v>
+      </x:c>
+      <x:c r="G14" s="3" t="str">
+        <x:v>Ask about fee assistance and funding referrals; no fee-waiver or cash commitment established</x:v>
+      </x:c>
+      <x:c r="H14" s="3" t="str">
+        <x:v>https://wsbdc.org/sbdc-services/</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="120" customHeight="1">
+      <x:c r="A15" s="3" t="str">
+        <x:v>Lynette / Business Impact NW</x:v>
+      </x:c>
+      <x:c r="B15" s="3" t="str">
+        <x:v>Free coaching and resource referrals</x:v>
+      </x:c>
+      <x:c r="C15" s="3" t="str">
+        <x:v>Existing free coaching</x:v>
+      </x:c>
+      <x:c r="D15" s="3" t="str">
+        <x:v>Coaching, not cash award</x:v>
+      </x:c>
+      <x:c r="E15" s="3" t="str">
+        <x:v>Orientation / program steps and appointment</x:v>
+      </x:c>
+      <x:c r="F15" s="3" t="str">
+        <x:v>Existing relationship; legal referral reply pending</x:v>
+      </x:c>
+      <x:c r="G15" s="3" t="str">
+        <x:v>Use Tuesday orientation and existing correspondence; do not duplicate coach setup</x:v>
+      </x:c>
+      <x:c r="H15" s="3" t="str">
+        <x:v>https://businessimpactnw.org/grow-your-business/coaching/</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="1"/>
+      <x:c r="B16" s="1"/>
+      <x:c r="C16" s="1"/>
+      <x:c r="D16" s="1"/>
+      <x:c r="E16" s="1"/>
+      <x:c r="F16" s="1"/>
+      <x:c r="G16" s="1"/>
+      <x:c r="H16" s="1"/>
+    </x:row>
+    <x:row r="17" ht="34" customHeight="1">
+      <x:c r="A17" s="3" t="str">
+        <x:v>TILE does not pay patent filing fees. SPL legal consults do not review documents. Seattle ABC requires an active city license.</x:v>
+      </x:c>
+      <x:c r="B17" s="3"/>
+      <x:c r="C17" s="3"/>
+      <x:c r="D17" s="3"/>
+      <x:c r="E17" s="3"/>
+      <x:c r="F17" s="3"/>
+      <x:c r="G17" s="3"/>
+      <x:c r="H17" s="3"/>
+    </x:row>
+    <x:row r="18" ht="34" customHeight="1">
+      <x:c r="A18" s="3" t="str">
+        <x:v>No loan-based capital program or reimbursement-only storefront fund is counted as cash available for this software/service launch.</x:v>
+      </x:c>
+      <x:c r="B18" s="3"/>
+      <x:c r="C18" s="3"/>
+      <x:c r="D18" s="3"/>
+      <x:c r="E18" s="3"/>
+      <x:c r="F18" s="3"/>
+      <x:c r="G18" s="3"/>
+      <x:c r="H18" s="3"/>
+    </x:row>
+    <x:row r="19" ht="34" customHeight="1">
+      <x:c r="A19" s="3" t="str">
+        <x:v>Only record a reduction after actual written acceptance covers the expense, or unrestricted usable grant funds are actually received.</x:v>
+      </x:c>
+      <x:c r="B19" s="3"/>
+      <x:c r="C19" s="3"/>
+      <x:c r="D19" s="3"/>
+      <x:c r="E19" s="3"/>
+      <x:c r="F19" s="3"/>
+      <x:c r="G19" s="3"/>
+      <x:c r="H19" s="3"/>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="1"/>
+      <x:c r="B20" s="1"/>
+      <x:c r="C20" s="1"/>
+      <x:c r="D20" s="1"/>
+      <x:c r="E20" s="1"/>
+      <x:c r="F20" s="1"/>
+      <x:c r="G20" s="1"/>
+      <x:c r="H20" s="1"/>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A3:H3"/>
+    <x:mergeCell ref="A4:H4"/>
+    <x:mergeCell ref="A17:H17"/>
+    <x:mergeCell ref="A18:H18"/>
+    <x:mergeCell ref="A19:H19"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
 </file>
</xml_diff>